<commit_message>
add visu for separate deflection system. missing alarm list
</commit_message>
<xml_diff>
--- a/4-3776/protocols/4-3776-communication-protocol-1.0.0.xlsx
+++ b/4-3776/protocols/4-3776-communication-protocol-1.0.0.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/kordianpiduch/Desktop/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{762B7B8C-8B09-2346-BD5B-FBF6173DACB7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{0956BA69-07B1-F445-A092-2BA2C065D439}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="2640" yWindow="960" windowWidth="37880" windowHeight="28400" tabRatio="713" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="12140" yWindow="1560" windowWidth="37880" windowHeight="28400" tabRatio="713" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="General Information" sheetId="1" r:id="rId1"/>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1331" uniqueCount="246">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1331" uniqueCount="179">
   <si>
     <t>ITEM</t>
   </si>
@@ -571,208 +571,7 @@
     <t>192.168.10.10/20</t>
   </si>
   <si>
-    <t>192.168.10.10/21</t>
-  </si>
-  <si>
-    <t>192.168.10.10/22</t>
-  </si>
-  <si>
-    <t>192.168.10.10/23</t>
-  </si>
-  <si>
-    <t>192.168.10.10/24</t>
-  </si>
-  <si>
-    <t>192.168.10.10/25</t>
-  </si>
-  <si>
-    <t>192.168.10.10/26</t>
-  </si>
-  <si>
-    <t>192.168.10.10/27</t>
-  </si>
-  <si>
-    <t>192.168.10.10/28</t>
-  </si>
-  <si>
-    <t>192.168.10.10/29</t>
-  </si>
-  <si>
-    <t>192.168.10.10/30</t>
-  </si>
-  <si>
-    <t>192.168.10.10/31</t>
-  </si>
-  <si>
-    <t>192.168.10.10/32</t>
-  </si>
-  <si>
-    <t>192.168.10.10/33</t>
-  </si>
-  <si>
-    <t>192.168.10.10/34</t>
-  </si>
-  <si>
-    <t>192.168.10.10/35</t>
-  </si>
-  <si>
-    <t>192.168.10.10/36</t>
-  </si>
-  <si>
-    <t>192.168.10.10/37</t>
-  </si>
-  <si>
-    <t>192.168.10.10/38</t>
-  </si>
-  <si>
-    <t>192.168.10.10/39</t>
-  </si>
-  <si>
-    <t>192.168.10.10/40</t>
-  </si>
-  <si>
-    <t>192.168.10.10/41</t>
-  </si>
-  <si>
-    <t>192.168.10.10/42</t>
-  </si>
-  <si>
-    <t>192.168.10.10/43</t>
-  </si>
-  <si>
-    <t>192.168.10.10/44</t>
-  </si>
-  <si>
-    <t>192.168.10.10/45</t>
-  </si>
-  <si>
-    <t>192.168.10.10/46</t>
-  </si>
-  <si>
-    <t>192.168.10.10/47</t>
-  </si>
-  <si>
-    <t>192.168.10.10/48</t>
-  </si>
-  <si>
-    <t>192.168.10.10/49</t>
-  </si>
-  <si>
-    <t>192.168.10.10/50</t>
-  </si>
-  <si>
-    <t>192.168.10.10/51</t>
-  </si>
-  <si>
-    <t>192.168.10.10/52</t>
-  </si>
-  <si>
-    <t>192.168.10.10/53</t>
-  </si>
-  <si>
-    <t>192.168.10.10/54</t>
-  </si>
-  <si>
-    <t>192.168.10.10/55</t>
-  </si>
-  <si>
-    <t>192.168.10.10/56</t>
-  </si>
-  <si>
-    <t>192.168.10.10/57</t>
-  </si>
-  <si>
-    <t>192.168.10.10/58</t>
-  </si>
-  <si>
-    <t>192.168.10.10/59</t>
-  </si>
-  <si>
-    <t>192.168.10.10/60</t>
-  </si>
-  <si>
-    <t>192.168.10.10/61</t>
-  </si>
-  <si>
-    <t>192.168.10.10/62</t>
-  </si>
-  <si>
-    <t>192.168.10.10/63</t>
-  </si>
-  <si>
-    <t>192.168.10.10/64</t>
-  </si>
-  <si>
-    <t>192.168.10.10/65</t>
-  </si>
-  <si>
-    <t>192.168.10.10/66</t>
-  </si>
-  <si>
-    <t>192.168.10.10/67</t>
-  </si>
-  <si>
-    <t>192.168.10.10/68</t>
-  </si>
-  <si>
-    <t>192.168.10.10/69</t>
-  </si>
-  <si>
-    <t>192.168.10.10/70</t>
-  </si>
-  <si>
-    <t>192.168.10.10/71</t>
-  </si>
-  <si>
-    <t>192.168.10.10/72</t>
-  </si>
-  <si>
-    <t>192.168.10.10/73</t>
-  </si>
-  <si>
-    <t>192.168.10.10/74</t>
-  </si>
-  <si>
-    <t>192.168.10.10/75</t>
-  </si>
-  <si>
-    <t>192.168.10.10/76</t>
-  </si>
-  <si>
-    <t>192.168.10.10/77</t>
-  </si>
-  <si>
-    <t>192.168.10.10/78</t>
-  </si>
-  <si>
-    <t>192.168.10.10/79</t>
-  </si>
-  <si>
-    <t>192.168.10.10/80</t>
-  </si>
-  <si>
-    <t>192.168.10.10/81</t>
-  </si>
-  <si>
-    <t>192.168.10.10/82</t>
-  </si>
-  <si>
-    <t>192.168.10.10/83</t>
-  </si>
-  <si>
-    <t>192.168.10.10/84</t>
-  </si>
-  <si>
-    <t>192.168.10.10/85</t>
-  </si>
-  <si>
-    <t>192.168.10.10/86</t>
-  </si>
-  <si>
-    <t>192.168.10.10/87</t>
-  </si>
-  <si>
-    <t>192.168.10.10/88</t>
+    <t>unit in control</t>
   </si>
 </sst>
 </file>
@@ -909,7 +708,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="22">
+  <borders count="23">
     <border>
       <left/>
       <right/>
@@ -1154,11 +953,20 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="thin">
+        <color theme="4" tint="0.39997558519241921"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="54">
+  <cellXfs count="53">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -1190,6 +998,36 @@
     <xf numFmtId="0" fontId="8" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="13" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="2" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="18" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="13" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="18" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="21" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="17" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -1201,6 +1039,27 @@
     </xf>
     <xf numFmtId="14" fontId="1" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -1223,30 +1082,6 @@
     <xf numFmtId="0" fontId="7" fillId="6" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="6" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="6" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -1262,14 +1097,20 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center"/>
+    <xf numFmtId="0" fontId="7" fillId="6" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="0" fontId="7" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="5" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="5" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="3" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -1280,44 +1121,8 @@
     <xf numFmtId="0" fontId="5" fillId="3" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="0" fillId="0" borderId="13" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="22" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="5" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="5" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="2" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1359,6 +1164,26 @@
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <border outline="0">
+        <top style="thin">
+          <color theme="4" tint="0.39997558519241921"/>
+        </top>
+      </border>
+    </dxf>
+    <dxf>
+      <border outline="0">
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
       <font>
         <b/>
         <i val="0"/>
@@ -1395,24 +1220,7 @@
       </border>
     </dxf>
     <dxf>
-      <border outline="0">
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <border outline="0">
-        <top style="thin">
-          <color theme="4" tint="0.39997558519241921"/>
-        </top>
-      </border>
     </dxf>
     <dxf>
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
@@ -1447,9 +1255,6 @@
           <color rgb="FF000000"/>
         </bottom>
       </border>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
       <fill>
@@ -1688,29 +1493,29 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{BCCC0CDB-2579-4D5D-B5F0-E975F3BF74E6}" name="Tabela22345" displayName="Tabela22345" ref="A4:I73" totalsRowShown="0" headerRowDxfId="23" dataDxfId="22" headerRowBorderDxfId="21">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{BCCC0CDB-2579-4D5D-B5F0-E975F3BF74E6}" name="Tabela22345" displayName="Tabela22345" ref="A4:I73" totalsRowShown="0" headerRowDxfId="23" dataDxfId="21" headerRowBorderDxfId="22">
   <autoFilter ref="A4:I73" xr:uid="{2F076FCC-5C32-47D1-A571-BDE4288C74C6}"/>
   <tableColumns count="9">
-    <tableColumn id="11" xr3:uid="{E20BFEB6-2D63-4482-90C1-A8967C3F1A6E}" name="PLC Modbus Slave Address" dataDxfId="13"/>
-    <tableColumn id="1" xr3:uid="{D2BC299D-ACA1-4C75-A6AF-05F2DC2E45FA}" name="Cabinet" dataDxfId="12"/>
-    <tableColumn id="3" xr3:uid="{FAFC91F5-A9CB-4426-B99B-8967122FF090}" name="Signal Type" dataDxfId="20"/>
-    <tableColumn id="4" xr3:uid="{4875BB2D-2846-4EC9-BD7B-ED58BD14C763}" name="Description" dataDxfId="19"/>
-    <tableColumn id="10" xr3:uid="{377896FA-D093-4616-A89B-19E84EA3F810}" name="Parameter" dataDxfId="18"/>
-    <tableColumn id="5" xr3:uid="{6EEA593A-47AC-4CBA-BD0E-A940F7B7634F}" name="Modbus Address" dataDxfId="17"/>
-    <tableColumn id="8" xr3:uid="{7ABF8B6A-E003-4247-AA13-4F093D0BA660}" name="Bit" dataDxfId="16"/>
-    <tableColumn id="7" xr3:uid="{4B08EF8A-9A9A-4DC6-BA17-FEBBE82E51BD}" name="Function Code" dataDxfId="15"/>
-    <tableColumn id="6" xr3:uid="{C43B2C1A-F284-4855-A1B6-5E2ACBF6BCBE}" name="Notes" dataDxfId="14"/>
+    <tableColumn id="11" xr3:uid="{E20BFEB6-2D63-4482-90C1-A8967C3F1A6E}" name="PLC Modbus Slave Address" dataDxfId="20"/>
+    <tableColumn id="1" xr3:uid="{D2BC299D-ACA1-4C75-A6AF-05F2DC2E45FA}" name="Cabinet" dataDxfId="19"/>
+    <tableColumn id="3" xr3:uid="{FAFC91F5-A9CB-4426-B99B-8967122FF090}" name="Signal Type" dataDxfId="18"/>
+    <tableColumn id="4" xr3:uid="{4875BB2D-2846-4EC9-BD7B-ED58BD14C763}" name="Description" dataDxfId="17"/>
+    <tableColumn id="10" xr3:uid="{377896FA-D093-4616-A89B-19E84EA3F810}" name="Parameter" dataDxfId="16"/>
+    <tableColumn id="5" xr3:uid="{6EEA593A-47AC-4CBA-BD0E-A940F7B7634F}" name="Modbus Address" dataDxfId="15"/>
+    <tableColumn id="8" xr3:uid="{7ABF8B6A-E003-4247-AA13-4F093D0BA660}" name="Bit" dataDxfId="14"/>
+    <tableColumn id="7" xr3:uid="{4B08EF8A-9A9A-4DC6-BA17-FEBBE82E51BD}" name="Function Code" dataDxfId="13"/>
+    <tableColumn id="6" xr3:uid="{C43B2C1A-F284-4855-A1B6-5E2ACBF6BCBE}" name="Notes" dataDxfId="12"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{81CFC7F6-4616-BC40-9808-DBECEF9D154B}" name="Table1" displayName="Table1" ref="A75:I107" totalsRowShown="0" headerRowDxfId="7" headerRowBorderDxfId="8" tableBorderDxfId="11">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{81CFC7F6-4616-BC40-9808-DBECEF9D154B}" name="Table1" displayName="Table1" ref="A75:I107" totalsRowShown="0" headerRowDxfId="11" headerRowBorderDxfId="10" tableBorderDxfId="9">
   <autoFilter ref="A75:I107" xr:uid="{81CFC7F6-4616-BC40-9808-DBECEF9D154B}"/>
   <tableColumns count="9">
-    <tableColumn id="1" xr3:uid="{DDAD954D-FCEF-E949-BC80-B1FCF4624024}" name="PLC Modbus Slave Address" dataDxfId="10"/>
-    <tableColumn id="2" xr3:uid="{037ABCB9-13C8-044F-8510-A0235A97102A}" name="Cabinet" dataDxfId="9"/>
+    <tableColumn id="1" xr3:uid="{DDAD954D-FCEF-E949-BC80-B1FCF4624024}" name="PLC Modbus Slave Address" dataDxfId="8"/>
+    <tableColumn id="2" xr3:uid="{037ABCB9-13C8-044F-8510-A0235A97102A}" name="Cabinet" dataDxfId="7"/>
     <tableColumn id="3" xr3:uid="{35435514-654A-0B4B-97CC-BC2B0FFF10AB}" name="Signal Type" dataDxfId="6"/>
     <tableColumn id="4" xr3:uid="{E4192124-0E92-9F4F-906F-BF6C03BC78C7}" name="Description" dataDxfId="5"/>
     <tableColumn id="5" xr3:uid="{D30EE95A-D0A7-114F-8801-CD7CBE0BD7D7}" name="Parameter" dataDxfId="4"/>
@@ -2057,282 +1862,282 @@
       <c r="C9" s="8" t="s">
         <v>5</v>
       </c>
-      <c r="D9" s="21" t="s">
+      <c r="D9" s="38" t="s">
         <v>6</v>
       </c>
-      <c r="E9" s="22"/>
-      <c r="F9" s="22"/>
-      <c r="G9" s="22"/>
-      <c r="H9" s="22"/>
-      <c r="I9" s="22"/>
-      <c r="J9" s="22"/>
-      <c r="K9" s="23"/>
-      <c r="L9" s="21" t="s">
+      <c r="E9" s="44"/>
+      <c r="F9" s="44"/>
+      <c r="G9" s="44"/>
+      <c r="H9" s="44"/>
+      <c r="I9" s="44"/>
+      <c r="J9" s="44"/>
+      <c r="K9" s="45"/>
+      <c r="L9" s="38" t="s">
         <v>7</v>
       </c>
-      <c r="M9" s="30"/>
+      <c r="M9" s="39"/>
     </row>
     <row r="10" spans="2:13" x14ac:dyDescent="0.2">
-      <c r="B10" s="11" t="s">
+      <c r="B10" s="21" t="s">
         <v>8</v>
       </c>
-      <c r="C10" s="13"/>
-      <c r="D10" s="15"/>
-      <c r="E10" s="16"/>
-      <c r="F10" s="16"/>
-      <c r="G10" s="16"/>
-      <c r="H10" s="16"/>
-      <c r="I10" s="16"/>
-      <c r="J10" s="16"/>
-      <c r="K10" s="17"/>
-      <c r="L10" s="31"/>
-      <c r="M10" s="32"/>
+      <c r="C10" s="23"/>
+      <c r="D10" s="32"/>
+      <c r="E10" s="33"/>
+      <c r="F10" s="33"/>
+      <c r="G10" s="33"/>
+      <c r="H10" s="33"/>
+      <c r="I10" s="33"/>
+      <c r="J10" s="33"/>
+      <c r="K10" s="34"/>
+      <c r="L10" s="40"/>
+      <c r="M10" s="41"/>
     </row>
     <row r="11" spans="2:13" ht="16" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="B11" s="12"/>
-      <c r="C11" s="14"/>
-      <c r="D11" s="18"/>
-      <c r="E11" s="19"/>
-      <c r="F11" s="19"/>
-      <c r="G11" s="19"/>
-      <c r="H11" s="19"/>
-      <c r="I11" s="19"/>
-      <c r="J11" s="19"/>
-      <c r="K11" s="20"/>
-      <c r="L11" s="33"/>
-      <c r="M11" s="34"/>
+      <c r="B11" s="22"/>
+      <c r="C11" s="24"/>
+      <c r="D11" s="35"/>
+      <c r="E11" s="36"/>
+      <c r="F11" s="36"/>
+      <c r="G11" s="36"/>
+      <c r="H11" s="36"/>
+      <c r="I11" s="36"/>
+      <c r="J11" s="36"/>
+      <c r="K11" s="37"/>
+      <c r="L11" s="42"/>
+      <c r="M11" s="43"/>
     </row>
     <row r="12" spans="2:13" x14ac:dyDescent="0.2">
-      <c r="B12" s="11" t="s">
+      <c r="B12" s="21" t="s">
         <v>9</v>
       </c>
-      <c r="C12" s="13"/>
-      <c r="D12" s="15"/>
-      <c r="E12" s="16"/>
-      <c r="F12" s="16"/>
-      <c r="G12" s="16"/>
-      <c r="H12" s="16"/>
-      <c r="I12" s="16"/>
-      <c r="J12" s="16"/>
-      <c r="K12" s="17"/>
-      <c r="L12" s="31"/>
-      <c r="M12" s="32"/>
+      <c r="C12" s="23"/>
+      <c r="D12" s="32"/>
+      <c r="E12" s="33"/>
+      <c r="F12" s="33"/>
+      <c r="G12" s="33"/>
+      <c r="H12" s="33"/>
+      <c r="I12" s="33"/>
+      <c r="J12" s="33"/>
+      <c r="K12" s="34"/>
+      <c r="L12" s="40"/>
+      <c r="M12" s="41"/>
     </row>
     <row r="13" spans="2:13" ht="16" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="B13" s="12"/>
-      <c r="C13" s="14"/>
-      <c r="D13" s="18"/>
-      <c r="E13" s="19"/>
-      <c r="F13" s="19"/>
-      <c r="G13" s="19"/>
-      <c r="H13" s="19"/>
-      <c r="I13" s="19"/>
-      <c r="J13" s="19"/>
-      <c r="K13" s="20"/>
-      <c r="L13" s="33"/>
-      <c r="M13" s="34"/>
+      <c r="B13" s="22"/>
+      <c r="C13" s="24"/>
+      <c r="D13" s="35"/>
+      <c r="E13" s="36"/>
+      <c r="F13" s="36"/>
+      <c r="G13" s="36"/>
+      <c r="H13" s="36"/>
+      <c r="I13" s="36"/>
+      <c r="J13" s="36"/>
+      <c r="K13" s="37"/>
+      <c r="L13" s="42"/>
+      <c r="M13" s="43"/>
     </row>
     <row r="14" spans="2:13" x14ac:dyDescent="0.2">
-      <c r="B14" s="11" t="s">
+      <c r="B14" s="21" t="s">
         <v>10</v>
       </c>
-      <c r="C14" s="13"/>
-      <c r="D14" s="15"/>
-      <c r="E14" s="16"/>
-      <c r="F14" s="16"/>
-      <c r="G14" s="16"/>
-      <c r="H14" s="16"/>
-      <c r="I14" s="16"/>
-      <c r="J14" s="16"/>
-      <c r="K14" s="17"/>
+      <c r="C14" s="23"/>
+      <c r="D14" s="32"/>
+      <c r="E14" s="33"/>
+      <c r="F14" s="33"/>
+      <c r="G14" s="33"/>
+      <c r="H14" s="33"/>
+      <c r="I14" s="33"/>
+      <c r="J14" s="33"/>
+      <c r="K14" s="34"/>
       <c r="L14" s="26"/>
       <c r="M14" s="27"/>
     </row>
     <row r="15" spans="2:13" ht="16" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="B15" s="12"/>
-      <c r="C15" s="14"/>
-      <c r="D15" s="18"/>
-      <c r="E15" s="19"/>
-      <c r="F15" s="19"/>
-      <c r="G15" s="19"/>
-      <c r="H15" s="19"/>
-      <c r="I15" s="19"/>
-      <c r="J15" s="19"/>
-      <c r="K15" s="20"/>
+      <c r="B15" s="22"/>
+      <c r="C15" s="24"/>
+      <c r="D15" s="35"/>
+      <c r="E15" s="36"/>
+      <c r="F15" s="36"/>
+      <c r="G15" s="36"/>
+      <c r="H15" s="36"/>
+      <c r="I15" s="36"/>
+      <c r="J15" s="36"/>
+      <c r="K15" s="37"/>
       <c r="L15" s="28"/>
       <c r="M15" s="29"/>
     </row>
     <row r="16" spans="2:13" x14ac:dyDescent="0.2">
-      <c r="B16" s="11" t="s">
+      <c r="B16" s="21" t="s">
         <v>11</v>
       </c>
-      <c r="C16" s="11"/>
-      <c r="D16" s="15"/>
-      <c r="E16" s="16"/>
-      <c r="F16" s="16"/>
-      <c r="G16" s="16"/>
-      <c r="H16" s="16"/>
-      <c r="I16" s="16"/>
-      <c r="J16" s="16"/>
-      <c r="K16" s="17"/>
+      <c r="C16" s="21"/>
+      <c r="D16" s="32"/>
+      <c r="E16" s="33"/>
+      <c r="F16" s="33"/>
+      <c r="G16" s="33"/>
+      <c r="H16" s="33"/>
+      <c r="I16" s="33"/>
+      <c r="J16" s="33"/>
+      <c r="K16" s="34"/>
       <c r="L16" s="26"/>
       <c r="M16" s="27"/>
     </row>
     <row r="17" spans="2:24" ht="16" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="B17" s="12"/>
-      <c r="C17" s="12"/>
-      <c r="D17" s="18"/>
-      <c r="E17" s="19"/>
-      <c r="F17" s="19"/>
-      <c r="G17" s="19"/>
-      <c r="H17" s="19"/>
-      <c r="I17" s="19"/>
-      <c r="J17" s="19"/>
-      <c r="K17" s="20"/>
+      <c r="B17" s="22"/>
+      <c r="C17" s="22"/>
+      <c r="D17" s="35"/>
+      <c r="E17" s="36"/>
+      <c r="F17" s="36"/>
+      <c r="G17" s="36"/>
+      <c r="H17" s="36"/>
+      <c r="I17" s="36"/>
+      <c r="J17" s="36"/>
+      <c r="K17" s="37"/>
       <c r="L17" s="28"/>
       <c r="M17" s="29"/>
     </row>
     <row r="18" spans="2:24" x14ac:dyDescent="0.2">
-      <c r="B18" s="11" t="s">
+      <c r="B18" s="21" t="s">
         <v>12</v>
       </c>
-      <c r="C18" s="11"/>
-      <c r="D18" s="15"/>
-      <c r="E18" s="16"/>
-      <c r="F18" s="16"/>
-      <c r="G18" s="16"/>
-      <c r="H18" s="16"/>
-      <c r="I18" s="16"/>
-      <c r="J18" s="16"/>
-      <c r="K18" s="17"/>
+      <c r="C18" s="21"/>
+      <c r="D18" s="32"/>
+      <c r="E18" s="33"/>
+      <c r="F18" s="33"/>
+      <c r="G18" s="33"/>
+      <c r="H18" s="33"/>
+      <c r="I18" s="33"/>
+      <c r="J18" s="33"/>
+      <c r="K18" s="34"/>
       <c r="L18" s="26"/>
       <c r="M18" s="27"/>
     </row>
     <row r="19" spans="2:24" ht="16" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="B19" s="12"/>
-      <c r="C19" s="12"/>
-      <c r="D19" s="18"/>
-      <c r="E19" s="19"/>
-      <c r="F19" s="19"/>
-      <c r="G19" s="19"/>
-      <c r="H19" s="19"/>
-      <c r="I19" s="19"/>
-      <c r="J19" s="19"/>
-      <c r="K19" s="20"/>
+      <c r="B19" s="22"/>
+      <c r="C19" s="22"/>
+      <c r="D19" s="35"/>
+      <c r="E19" s="36"/>
+      <c r="F19" s="36"/>
+      <c r="G19" s="36"/>
+      <c r="H19" s="36"/>
+      <c r="I19" s="36"/>
+      <c r="J19" s="36"/>
+      <c r="K19" s="37"/>
       <c r="L19" s="28"/>
       <c r="M19" s="29"/>
     </row>
     <row r="20" spans="2:24" x14ac:dyDescent="0.2">
-      <c r="B20" s="11" t="s">
+      <c r="B20" s="21" t="s">
         <v>13</v>
       </c>
-      <c r="C20" s="11"/>
-      <c r="D20" s="15"/>
-      <c r="E20" s="16"/>
-      <c r="F20" s="16"/>
-      <c r="G20" s="16"/>
-      <c r="H20" s="16"/>
-      <c r="I20" s="16"/>
-      <c r="J20" s="16"/>
-      <c r="K20" s="17"/>
+      <c r="C20" s="21"/>
+      <c r="D20" s="32"/>
+      <c r="E20" s="33"/>
+      <c r="F20" s="33"/>
+      <c r="G20" s="33"/>
+      <c r="H20" s="33"/>
+      <c r="I20" s="33"/>
+      <c r="J20" s="33"/>
+      <c r="K20" s="34"/>
       <c r="L20" s="26"/>
       <c r="M20" s="27"/>
     </row>
     <row r="21" spans="2:24" ht="16" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="B21" s="12"/>
-      <c r="C21" s="12"/>
-      <c r="D21" s="18"/>
-      <c r="E21" s="19"/>
-      <c r="F21" s="19"/>
-      <c r="G21" s="19"/>
-      <c r="H21" s="19"/>
-      <c r="I21" s="19"/>
-      <c r="J21" s="19"/>
-      <c r="K21" s="20"/>
+      <c r="B21" s="22"/>
+      <c r="C21" s="22"/>
+      <c r="D21" s="35"/>
+      <c r="E21" s="36"/>
+      <c r="F21" s="36"/>
+      <c r="G21" s="36"/>
+      <c r="H21" s="36"/>
+      <c r="I21" s="36"/>
+      <c r="J21" s="36"/>
+      <c r="K21" s="37"/>
       <c r="L21" s="28"/>
       <c r="M21" s="29"/>
     </row>
     <row r="22" spans="2:24" x14ac:dyDescent="0.2">
-      <c r="B22" s="11" t="s">
+      <c r="B22" s="21" t="s">
         <v>14</v>
       </c>
-      <c r="C22" s="11"/>
-      <c r="D22" s="15"/>
-      <c r="E22" s="16"/>
-      <c r="F22" s="16"/>
-      <c r="G22" s="16"/>
-      <c r="H22" s="16"/>
-      <c r="I22" s="16"/>
-      <c r="J22" s="16"/>
-      <c r="K22" s="17"/>
+      <c r="C22" s="21"/>
+      <c r="D22" s="32"/>
+      <c r="E22" s="33"/>
+      <c r="F22" s="33"/>
+      <c r="G22" s="33"/>
+      <c r="H22" s="33"/>
+      <c r="I22" s="33"/>
+      <c r="J22" s="33"/>
+      <c r="K22" s="34"/>
       <c r="L22" s="26"/>
       <c r="M22" s="27"/>
     </row>
     <row r="23" spans="2:24" ht="16" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="B23" s="12"/>
-      <c r="C23" s="12"/>
-      <c r="D23" s="18"/>
-      <c r="E23" s="19"/>
-      <c r="F23" s="19"/>
-      <c r="G23" s="19"/>
-      <c r="H23" s="19"/>
-      <c r="I23" s="19"/>
-      <c r="J23" s="19"/>
-      <c r="K23" s="20"/>
+      <c r="B23" s="22"/>
+      <c r="C23" s="22"/>
+      <c r="D23" s="35"/>
+      <c r="E23" s="36"/>
+      <c r="F23" s="36"/>
+      <c r="G23" s="36"/>
+      <c r="H23" s="36"/>
+      <c r="I23" s="36"/>
+      <c r="J23" s="36"/>
+      <c r="K23" s="37"/>
       <c r="L23" s="28"/>
       <c r="M23" s="29"/>
     </row>
     <row r="26" spans="2:24" x14ac:dyDescent="0.2">
-      <c r="B26" s="36" t="s">
+      <c r="B26" s="25" t="s">
         <v>20</v>
       </c>
-      <c r="C26" s="36"/>
-      <c r="D26" s="36"/>
-      <c r="E26" s="36"/>
-      <c r="F26" s="36"/>
-      <c r="G26" s="36"/>
-      <c r="H26" s="36"/>
-      <c r="I26" s="36"/>
-      <c r="J26" s="36"/>
-      <c r="K26" s="36"/>
-      <c r="L26" s="36"/>
-      <c r="M26" s="36"/>
-      <c r="N26" s="36"/>
-      <c r="O26" s="36"/>
-      <c r="P26" s="36"/>
-      <c r="Q26" s="36"/>
-      <c r="R26" s="36"/>
-      <c r="S26" s="36"/>
-      <c r="T26" s="36"/>
-      <c r="U26" s="36"/>
-      <c r="V26" s="36"/>
-      <c r="W26" s="36"/>
-      <c r="X26" s="36"/>
+      <c r="C26" s="25"/>
+      <c r="D26" s="25"/>
+      <c r="E26" s="25"/>
+      <c r="F26" s="25"/>
+      <c r="G26" s="25"/>
+      <c r="H26" s="25"/>
+      <c r="I26" s="25"/>
+      <c r="J26" s="25"/>
+      <c r="K26" s="25"/>
+      <c r="L26" s="25"/>
+      <c r="M26" s="25"/>
+      <c r="N26" s="25"/>
+      <c r="O26" s="25"/>
+      <c r="P26" s="25"/>
+      <c r="Q26" s="25"/>
+      <c r="R26" s="25"/>
+      <c r="S26" s="25"/>
+      <c r="T26" s="25"/>
+      <c r="U26" s="25"/>
+      <c r="V26" s="25"/>
+      <c r="W26" s="25"/>
+      <c r="X26" s="25"/>
     </row>
     <row r="27" spans="2:24" x14ac:dyDescent="0.2">
-      <c r="B27" s="36"/>
-      <c r="C27" s="36"/>
-      <c r="D27" s="36"/>
-      <c r="E27" s="36"/>
-      <c r="F27" s="36"/>
-      <c r="G27" s="36"/>
-      <c r="H27" s="36"/>
-      <c r="I27" s="36"/>
-      <c r="J27" s="36"/>
-      <c r="K27" s="36"/>
-      <c r="L27" s="36"/>
-      <c r="M27" s="36"/>
-      <c r="N27" s="36"/>
-      <c r="O27" s="36"/>
-      <c r="P27" s="36"/>
-      <c r="Q27" s="36"/>
-      <c r="R27" s="36"/>
-      <c r="S27" s="36"/>
-      <c r="T27" s="36"/>
-      <c r="U27" s="36"/>
-      <c r="V27" s="36"/>
-      <c r="W27" s="36"/>
-      <c r="X27" s="36"/>
+      <c r="B27" s="25"/>
+      <c r="C27" s="25"/>
+      <c r="D27" s="25"/>
+      <c r="E27" s="25"/>
+      <c r="F27" s="25"/>
+      <c r="G27" s="25"/>
+      <c r="H27" s="25"/>
+      <c r="I27" s="25"/>
+      <c r="J27" s="25"/>
+      <c r="K27" s="25"/>
+      <c r="L27" s="25"/>
+      <c r="M27" s="25"/>
+      <c r="N27" s="25"/>
+      <c r="O27" s="25"/>
+      <c r="P27" s="25"/>
+      <c r="Q27" s="25"/>
+      <c r="R27" s="25"/>
+      <c r="S27" s="25"/>
+      <c r="T27" s="25"/>
+      <c r="U27" s="25"/>
+      <c r="V27" s="25"/>
+      <c r="W27" s="25"/>
+      <c r="X27" s="25"/>
     </row>
     <row r="29" spans="2:24" x14ac:dyDescent="0.2">
       <c r="B29" t="s">
@@ -2341,8 +2146,8 @@
     </row>
     <row r="30" spans="2:24" x14ac:dyDescent="0.2">
       <c r="B30" s="2"/>
-      <c r="C30" s="35"/>
-      <c r="D30" s="35"/>
+      <c r="C30" s="20"/>
+      <c r="D30" s="20"/>
     </row>
     <row r="31" spans="2:24" x14ac:dyDescent="0.2">
       <c r="B31" s="2" t="s">
@@ -2461,48 +2266,48 @@
       <c r="T44" s="1"/>
     </row>
     <row r="45" spans="1:21" x14ac:dyDescent="0.2">
-      <c r="B45" s="24"/>
-      <c r="C45" s="24"/>
-      <c r="D45" s="24"/>
-      <c r="E45" s="24"/>
-      <c r="F45" s="24"/>
-      <c r="G45" s="24"/>
-      <c r="H45" s="24"/>
-      <c r="I45" s="24"/>
-      <c r="J45" s="24"/>
-      <c r="K45" s="24"/>
-      <c r="L45" s="24"/>
-      <c r="M45" s="24"/>
-      <c r="N45" s="24"/>
-      <c r="O45" s="24"/>
-      <c r="P45" s="24"/>
-      <c r="Q45" s="24"/>
-      <c r="R45" s="24"/>
-      <c r="S45" s="24"/>
-      <c r="T45" s="24"/>
-      <c r="U45" s="24"/>
+      <c r="B45" s="30"/>
+      <c r="C45" s="30"/>
+      <c r="D45" s="30"/>
+      <c r="E45" s="30"/>
+      <c r="F45" s="30"/>
+      <c r="G45" s="30"/>
+      <c r="H45" s="30"/>
+      <c r="I45" s="30"/>
+      <c r="J45" s="30"/>
+      <c r="K45" s="30"/>
+      <c r="L45" s="30"/>
+      <c r="M45" s="30"/>
+      <c r="N45" s="30"/>
+      <c r="O45" s="30"/>
+      <c r="P45" s="30"/>
+      <c r="Q45" s="30"/>
+      <c r="R45" s="30"/>
+      <c r="S45" s="30"/>
+      <c r="T45" s="30"/>
+      <c r="U45" s="30"/>
     </row>
     <row r="47" spans="1:21" x14ac:dyDescent="0.2">
-      <c r="B47" s="25"/>
-      <c r="C47" s="25"/>
-      <c r="D47" s="25"/>
-      <c r="E47" s="25"/>
-      <c r="F47" s="25"/>
-      <c r="G47" s="25"/>
-      <c r="H47" s="25"/>
-      <c r="I47" s="25"/>
-      <c r="J47" s="25"/>
-      <c r="K47" s="25"/>
-      <c r="L47" s="25"/>
-      <c r="M47" s="25"/>
-      <c r="N47" s="25"/>
-      <c r="O47" s="25"/>
-      <c r="P47" s="25"/>
-      <c r="Q47" s="25"/>
-      <c r="R47" s="25"/>
-      <c r="S47" s="25"/>
-      <c r="T47" s="25"/>
-      <c r="U47" s="25"/>
+      <c r="B47" s="31"/>
+      <c r="C47" s="31"/>
+      <c r="D47" s="31"/>
+      <c r="E47" s="31"/>
+      <c r="F47" s="31"/>
+      <c r="G47" s="31"/>
+      <c r="H47" s="31"/>
+      <c r="I47" s="31"/>
+      <c r="J47" s="31"/>
+      <c r="K47" s="31"/>
+      <c r="L47" s="31"/>
+      <c r="M47" s="31"/>
+      <c r="N47" s="31"/>
+      <c r="O47" s="31"/>
+      <c r="P47" s="31"/>
+      <c r="Q47" s="31"/>
+      <c r="R47" s="31"/>
+      <c r="S47" s="31"/>
+      <c r="T47" s="31"/>
+      <c r="U47" s="31"/>
     </row>
     <row r="72" spans="21:24" x14ac:dyDescent="0.2">
       <c r="U72" s="1"/>
@@ -2527,17 +2332,13 @@
     <row r="97" ht="26.5" customHeight="1" x14ac:dyDescent="0.2"/>
   </sheetData>
   <mergeCells count="34">
-    <mergeCell ref="C30:D30"/>
-    <mergeCell ref="B14:B15"/>
-    <mergeCell ref="C14:C15"/>
-    <mergeCell ref="B16:B17"/>
-    <mergeCell ref="C16:C17"/>
-    <mergeCell ref="B26:X27"/>
-    <mergeCell ref="L20:M21"/>
-    <mergeCell ref="B18:B19"/>
-    <mergeCell ref="C18:C19"/>
-    <mergeCell ref="B20:B21"/>
-    <mergeCell ref="C20:C21"/>
+    <mergeCell ref="B10:B11"/>
+    <mergeCell ref="C10:C11"/>
+    <mergeCell ref="D18:K19"/>
+    <mergeCell ref="D20:K21"/>
+    <mergeCell ref="D9:K9"/>
+    <mergeCell ref="B12:B13"/>
+    <mergeCell ref="C12:C13"/>
     <mergeCell ref="B45:U45"/>
     <mergeCell ref="B47:U47"/>
     <mergeCell ref="L16:M17"/>
@@ -2554,13 +2355,17 @@
     <mergeCell ref="D10:K11"/>
     <mergeCell ref="D12:K13"/>
     <mergeCell ref="D14:K15"/>
-    <mergeCell ref="B10:B11"/>
-    <mergeCell ref="C10:C11"/>
-    <mergeCell ref="D18:K19"/>
-    <mergeCell ref="D20:K21"/>
-    <mergeCell ref="D9:K9"/>
-    <mergeCell ref="B12:B13"/>
-    <mergeCell ref="C12:C13"/>
+    <mergeCell ref="C30:D30"/>
+    <mergeCell ref="B14:B15"/>
+    <mergeCell ref="C14:C15"/>
+    <mergeCell ref="B16:B17"/>
+    <mergeCell ref="C16:C17"/>
+    <mergeCell ref="B26:X27"/>
+    <mergeCell ref="L20:M21"/>
+    <mergeCell ref="B18:B19"/>
+    <mergeCell ref="C18:C19"/>
+    <mergeCell ref="B20:B21"/>
+    <mergeCell ref="C20:C21"/>
   </mergeCells>
   <phoneticPr fontId="3" type="noConversion"/>
   <pageMargins left="0.19685039370078741" right="0.19685039370078741" top="0.74803149606299213" bottom="0.74803149606299213" header="0.31496062992125984" footer="0.31496062992125984"/>
@@ -2597,26 +2402,26 @@
   </cols>
   <sheetData>
     <row r="2" spans="1:9" ht="14.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A2" s="37"/>
-      <c r="B2" s="37"/>
-      <c r="C2" s="37"/>
-      <c r="D2" s="37"/>
-      <c r="E2" s="37"/>
-      <c r="F2" s="37"/>
-      <c r="G2" s="37"/>
-      <c r="H2" s="37"/>
-      <c r="I2" s="37"/>
+      <c r="A2" s="46"/>
+      <c r="B2" s="46"/>
+      <c r="C2" s="46"/>
+      <c r="D2" s="46"/>
+      <c r="E2" s="46"/>
+      <c r="F2" s="46"/>
+      <c r="G2" s="46"/>
+      <c r="H2" s="46"/>
+      <c r="I2" s="46"/>
     </row>
     <row r="3" spans="1:9" ht="14.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A3" s="37"/>
-      <c r="B3" s="37"/>
-      <c r="C3" s="37"/>
-      <c r="D3" s="37"/>
-      <c r="E3" s="37"/>
-      <c r="F3" s="37"/>
-      <c r="G3" s="37"/>
-      <c r="H3" s="37"/>
-      <c r="I3" s="37"/>
+      <c r="A3" s="46"/>
+      <c r="B3" s="46"/>
+      <c r="C3" s="46"/>
+      <c r="D3" s="46"/>
+      <c r="E3" s="46"/>
+      <c r="F3" s="46"/>
+      <c r="G3" s="46"/>
+      <c r="H3" s="46"/>
+      <c r="I3" s="46"/>
     </row>
     <row r="4" spans="1:9" ht="83" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A4" s="3" t="s">
@@ -8953,41 +8758,41 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:9" ht="14.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A1" s="38" t="s">
+      <c r="A1" s="49" t="s">
         <v>39</v>
       </c>
-      <c r="B1" s="44"/>
-      <c r="C1" s="44"/>
-      <c r="D1" s="44"/>
-      <c r="E1" s="44"/>
-      <c r="F1" s="44"/>
-      <c r="G1" s="44"/>
-      <c r="H1" s="44"/>
-      <c r="I1" s="44"/>
+      <c r="B1" s="46"/>
+      <c r="C1" s="46"/>
+      <c r="D1" s="46"/>
+      <c r="E1" s="46"/>
+      <c r="F1" s="46"/>
+      <c r="G1" s="46"/>
+      <c r="H1" s="46"/>
+      <c r="I1" s="46"/>
     </row>
     <row r="2" spans="1:9" ht="14.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A2" s="39"/>
-      <c r="B2" s="40"/>
-      <c r="C2" s="40"/>
-      <c r="D2" s="40"/>
-      <c r="E2" s="40"/>
-      <c r="F2" s="40"/>
-      <c r="G2" s="40"/>
-      <c r="H2" s="40"/>
-      <c r="I2" s="40"/>
+      <c r="A2" s="50"/>
+      <c r="B2" s="51"/>
+      <c r="C2" s="51"/>
+      <c r="D2" s="51"/>
+      <c r="E2" s="51"/>
+      <c r="F2" s="51"/>
+      <c r="G2" s="51"/>
+      <c r="H2" s="51"/>
+      <c r="I2" s="51"/>
     </row>
     <row r="3" spans="1:9" ht="29" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A3" s="45" t="s">
+      <c r="A3" s="47" t="s">
         <v>175</v>
       </c>
-      <c r="B3" s="46"/>
-      <c r="C3" s="46"/>
-      <c r="D3" s="46"/>
-      <c r="E3" s="46"/>
-      <c r="F3" s="46"/>
-      <c r="G3" s="46"/>
-      <c r="H3" s="46"/>
-      <c r="I3" s="46"/>
+      <c r="B3" s="48"/>
+      <c r="C3" s="48"/>
+      <c r="D3" s="48"/>
+      <c r="E3" s="48"/>
+      <c r="F3" s="48"/>
+      <c r="G3" s="48"/>
+      <c r="H3" s="48"/>
+      <c r="I3" s="48"/>
     </row>
     <row r="4" spans="1:9" ht="83" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A4" s="3" t="s">
@@ -9047,7 +8852,7 @@
     </row>
     <row r="6" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A6" s="2" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="B6" s="2"/>
       <c r="C6" s="2" t="s">
@@ -9074,7 +8879,7 @@
     </row>
     <row r="7" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A7" s="2" t="s">
-        <v>179</v>
+        <v>177</v>
       </c>
       <c r="B7" s="2"/>
       <c r="C7" s="2" t="s">
@@ -9101,7 +8906,7 @@
     </row>
     <row r="8" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A8" s="2" t="s">
-        <v>180</v>
+        <v>177</v>
       </c>
       <c r="B8" s="2"/>
       <c r="C8" s="2" t="s">
@@ -9128,7 +8933,7 @@
     </row>
     <row r="9" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A9" s="2" t="s">
-        <v>181</v>
+        <v>177</v>
       </c>
       <c r="B9" s="2"/>
       <c r="C9" s="2" t="s">
@@ -9155,7 +8960,7 @@
     </row>
     <row r="10" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A10" s="2" t="s">
-        <v>182</v>
+        <v>177</v>
       </c>
       <c r="B10" s="2"/>
       <c r="C10" s="2" t="s">
@@ -9182,7 +8987,7 @@
     </row>
     <row r="11" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A11" s="2" t="s">
-        <v>183</v>
+        <v>177</v>
       </c>
       <c r="B11" s="2"/>
       <c r="C11" s="2" t="s">
@@ -9209,7 +9014,7 @@
     </row>
     <row r="12" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A12" s="2" t="s">
-        <v>184</v>
+        <v>177</v>
       </c>
       <c r="B12" s="2"/>
       <c r="C12" s="2" t="s">
@@ -9236,7 +9041,7 @@
     </row>
     <row r="13" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A13" s="2" t="s">
-        <v>185</v>
+        <v>177</v>
       </c>
       <c r="B13" s="2"/>
       <c r="C13" s="2" t="s">
@@ -9263,7 +9068,7 @@
     </row>
     <row r="14" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A14" s="2" t="s">
-        <v>186</v>
+        <v>177</v>
       </c>
       <c r="B14" s="2"/>
       <c r="C14" s="2" t="s">
@@ -9290,7 +9095,7 @@
     </row>
     <row r="15" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A15" s="2" t="s">
-        <v>187</v>
+        <v>177</v>
       </c>
       <c r="B15" s="2"/>
       <c r="C15" s="2" t="s">
@@ -9317,7 +9122,7 @@
     </row>
     <row r="16" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A16" s="2" t="s">
-        <v>188</v>
+        <v>177</v>
       </c>
       <c r="B16" s="2"/>
       <c r="C16" s="2" t="s">
@@ -9344,7 +9149,7 @@
     </row>
     <row r="17" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A17" s="2" t="s">
-        <v>189</v>
+        <v>177</v>
       </c>
       <c r="B17" s="2"/>
       <c r="C17" s="2" t="s">
@@ -9371,7 +9176,7 @@
     </row>
     <row r="18" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A18" s="2" t="s">
-        <v>190</v>
+        <v>177</v>
       </c>
       <c r="B18" s="2"/>
       <c r="C18" s="2" t="s">
@@ -9398,7 +9203,7 @@
     </row>
     <row r="19" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A19" s="2" t="s">
-        <v>191</v>
+        <v>177</v>
       </c>
       <c r="B19" s="2"/>
       <c r="C19" s="2" t="s">
@@ -9425,7 +9230,7 @@
     </row>
     <row r="20" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A20" s="2" t="s">
-        <v>192</v>
+        <v>177</v>
       </c>
       <c r="B20" s="2"/>
       <c r="C20" s="2" t="s">
@@ -9452,7 +9257,7 @@
     </row>
     <row r="21" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A21" s="2" t="s">
-        <v>193</v>
+        <v>177</v>
       </c>
       <c r="B21" s="2"/>
       <c r="C21" s="2" t="s">
@@ -9479,7 +9284,7 @@
     </row>
     <row r="22" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A22" s="2" t="s">
-        <v>194</v>
+        <v>177</v>
       </c>
       <c r="B22" s="2"/>
       <c r="C22" s="2" t="s">
@@ -9506,7 +9311,7 @@
     </row>
     <row r="23" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A23" s="2" t="s">
-        <v>195</v>
+        <v>177</v>
       </c>
       <c r="B23" s="2"/>
       <c r="C23" s="2" t="s">
@@ -9533,7 +9338,7 @@
     </row>
     <row r="24" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A24" s="2" t="s">
-        <v>196</v>
+        <v>177</v>
       </c>
       <c r="B24" s="2"/>
       <c r="C24" s="2" t="s">
@@ -9560,7 +9365,7 @@
     </row>
     <row r="25" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A25" s="2" t="s">
-        <v>197</v>
+        <v>177</v>
       </c>
       <c r="B25" s="2"/>
       <c r="C25" s="2" t="s">
@@ -9587,7 +9392,7 @@
     </row>
     <row r="26" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A26" s="2" t="s">
-        <v>198</v>
+        <v>177</v>
       </c>
       <c r="B26" s="2"/>
       <c r="C26" s="2" t="s">
@@ -9614,7 +9419,7 @@
     </row>
     <row r="27" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A27" s="2" t="s">
-        <v>199</v>
+        <v>177</v>
       </c>
       <c r="B27" s="2"/>
       <c r="C27" s="2" t="s">
@@ -9641,7 +9446,7 @@
     </row>
     <row r="28" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A28" s="2" t="s">
-        <v>200</v>
+        <v>177</v>
       </c>
       <c r="B28" s="2"/>
       <c r="C28" s="2" t="s">
@@ -9668,7 +9473,7 @@
     </row>
     <row r="29" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A29" s="2" t="s">
-        <v>201</v>
+        <v>177</v>
       </c>
       <c r="B29" s="2"/>
       <c r="C29" s="2" t="s">
@@ -9695,7 +9500,7 @@
     </row>
     <row r="30" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A30" s="2" t="s">
-        <v>202</v>
+        <v>177</v>
       </c>
       <c r="B30" s="2"/>
       <c r="C30" s="2" t="s">
@@ -9722,7 +9527,7 @@
     </row>
     <row r="31" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A31" s="2" t="s">
-        <v>203</v>
+        <v>177</v>
       </c>
       <c r="B31" s="2"/>
       <c r="C31" s="2" t="s">
@@ -9749,7 +9554,7 @@
     </row>
     <row r="32" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A32" s="2" t="s">
-        <v>204</v>
+        <v>177</v>
       </c>
       <c r="B32" s="2"/>
       <c r="C32" s="2" t="s">
@@ -9776,7 +9581,7 @@
     </row>
     <row r="33" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A33" s="2" t="s">
-        <v>205</v>
+        <v>177</v>
       </c>
       <c r="B33" s="2"/>
       <c r="C33" s="2" t="s">
@@ -9803,7 +9608,7 @@
     </row>
     <row r="34" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A34" s="2" t="s">
-        <v>206</v>
+        <v>177</v>
       </c>
       <c r="B34" s="2"/>
       <c r="C34" s="2" t="s">
@@ -9830,7 +9635,7 @@
     </row>
     <row r="35" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A35" s="2" t="s">
-        <v>207</v>
+        <v>177</v>
       </c>
       <c r="B35" s="2"/>
       <c r="C35" s="2" t="s">
@@ -9857,7 +9662,7 @@
     </row>
     <row r="36" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A36" s="2" t="s">
-        <v>208</v>
+        <v>177</v>
       </c>
       <c r="B36" s="2"/>
       <c r="C36" s="2" t="s">
@@ -9884,7 +9689,7 @@
     </row>
     <row r="37" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A37" s="2" t="s">
-        <v>209</v>
+        <v>177</v>
       </c>
       <c r="B37" s="2"/>
       <c r="C37" s="2" t="s">
@@ -9911,7 +9716,7 @@
     </row>
     <row r="38" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A38" s="2" t="s">
-        <v>210</v>
+        <v>177</v>
       </c>
       <c r="B38" s="2"/>
       <c r="C38" s="2" t="s">
@@ -9938,7 +9743,7 @@
     </row>
     <row r="39" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A39" s="2" t="s">
-        <v>211</v>
+        <v>177</v>
       </c>
       <c r="B39" s="2"/>
       <c r="C39" s="2" t="s">
@@ -9965,7 +9770,7 @@
     </row>
     <row r="40" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A40" s="2" t="s">
-        <v>212</v>
+        <v>177</v>
       </c>
       <c r="B40" s="2"/>
       <c r="C40" s="2" t="s">
@@ -9992,7 +9797,7 @@
     </row>
     <row r="41" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A41" s="2" t="s">
-        <v>213</v>
+        <v>177</v>
       </c>
       <c r="B41" s="2"/>
       <c r="C41" s="2" t="s">
@@ -10019,7 +9824,7 @@
     </row>
     <row r="42" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A42" s="2" t="s">
-        <v>214</v>
+        <v>177</v>
       </c>
       <c r="B42" s="2"/>
       <c r="C42" s="2" t="s">
@@ -10046,7 +9851,7 @@
     </row>
     <row r="43" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A43" s="2" t="s">
-        <v>215</v>
+        <v>177</v>
       </c>
       <c r="B43" s="2"/>
       <c r="C43" s="2" t="s">
@@ -10073,7 +9878,7 @@
     </row>
     <row r="44" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A44" s="2" t="s">
-        <v>216</v>
+        <v>177</v>
       </c>
       <c r="B44" s="2"/>
       <c r="C44" s="2" t="s">
@@ -10100,7 +9905,7 @@
     </row>
     <row r="45" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A45" s="2" t="s">
-        <v>217</v>
+        <v>177</v>
       </c>
       <c r="B45" s="2"/>
       <c r="C45" s="2" t="s">
@@ -10127,7 +9932,7 @@
     </row>
     <row r="46" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A46" s="2" t="s">
-        <v>218</v>
+        <v>177</v>
       </c>
       <c r="B46" s="2"/>
       <c r="C46" s="2" t="s">
@@ -10154,7 +9959,7 @@
     </row>
     <row r="47" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A47" s="2" t="s">
-        <v>219</v>
+        <v>177</v>
       </c>
       <c r="B47" s="2"/>
       <c r="C47" s="2" t="s">
@@ -10181,7 +9986,7 @@
     </row>
     <row r="48" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A48" s="2" t="s">
-        <v>220</v>
+        <v>177</v>
       </c>
       <c r="B48" s="2"/>
       <c r="C48" s="2" t="s">
@@ -10208,7 +10013,7 @@
     </row>
     <row r="49" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A49" s="2" t="s">
-        <v>221</v>
+        <v>177</v>
       </c>
       <c r="B49" s="2"/>
       <c r="C49" s="2" t="s">
@@ -10235,7 +10040,7 @@
     </row>
     <row r="50" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A50" s="2" t="s">
-        <v>222</v>
+        <v>177</v>
       </c>
       <c r="B50" s="2"/>
       <c r="C50" s="2" t="s">
@@ -10262,7 +10067,7 @@
     </row>
     <row r="51" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A51" s="2" t="s">
-        <v>223</v>
+        <v>177</v>
       </c>
       <c r="B51" s="2"/>
       <c r="C51" s="2" t="s">
@@ -10289,7 +10094,7 @@
     </row>
     <row r="52" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A52" s="2" t="s">
-        <v>224</v>
+        <v>177</v>
       </c>
       <c r="B52" s="2"/>
       <c r="C52" s="2" t="s">
@@ -10316,7 +10121,7 @@
     </row>
     <row r="53" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A53" s="2" t="s">
-        <v>225</v>
+        <v>177</v>
       </c>
       <c r="B53" s="2"/>
       <c r="C53" s="2" t="s">
@@ -10325,7 +10130,7 @@
       <c r="D53" t="s">
         <v>125</v>
       </c>
-      <c r="E53" s="41" t="s">
+      <c r="E53" s="2" t="s">
         <v>38</v>
       </c>
       <c r="F53" s="2">
@@ -10343,7 +10148,7 @@
     </row>
     <row r="54" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A54" s="2" t="s">
-        <v>226</v>
+        <v>177</v>
       </c>
       <c r="B54" s="2"/>
       <c r="C54" s="2" t="s">
@@ -10352,7 +10157,7 @@
       <c r="D54" t="s">
         <v>126</v>
       </c>
-      <c r="E54" s="41" t="s">
+      <c r="E54" s="2" t="s">
         <v>38</v>
       </c>
       <c r="F54" s="2">
@@ -10370,7 +10175,7 @@
     </row>
     <row r="55" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A55" s="2" t="s">
-        <v>227</v>
+        <v>177</v>
       </c>
       <c r="B55" s="2"/>
       <c r="C55" s="2" t="s">
@@ -10379,7 +10184,7 @@
       <c r="D55" t="s">
         <v>127</v>
       </c>
-      <c r="E55" s="41" t="s">
+      <c r="E55" s="2" t="s">
         <v>38</v>
       </c>
       <c r="F55" s="2">
@@ -10397,7 +10202,7 @@
     </row>
     <row r="56" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A56" s="2" t="s">
-        <v>228</v>
+        <v>177</v>
       </c>
       <c r="B56" s="2"/>
       <c r="C56" s="2" t="s">
@@ -10406,7 +10211,7 @@
       <c r="D56" t="s">
         <v>128</v>
       </c>
-      <c r="E56" s="41" t="s">
+      <c r="E56" s="2" t="s">
         <v>38</v>
       </c>
       <c r="F56" s="2">
@@ -10424,7 +10229,7 @@
     </row>
     <row r="57" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A57" s="2" t="s">
-        <v>229</v>
+        <v>177</v>
       </c>
       <c r="B57" s="2"/>
       <c r="C57" s="2" t="s">
@@ -10433,7 +10238,7 @@
       <c r="D57" t="s">
         <v>129</v>
       </c>
-      <c r="E57" s="41" t="s">
+      <c r="E57" s="2" t="s">
         <v>38</v>
       </c>
       <c r="F57" s="2">
@@ -10451,7 +10256,7 @@
     </row>
     <row r="58" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A58" s="2" t="s">
-        <v>230</v>
+        <v>177</v>
       </c>
       <c r="B58" s="2"/>
       <c r="C58" s="2" t="s">
@@ -10460,7 +10265,7 @@
       <c r="D58" t="s">
         <v>130</v>
       </c>
-      <c r="E58" s="41" t="s">
+      <c r="E58" s="2" t="s">
         <v>38</v>
       </c>
       <c r="F58" s="2">
@@ -10478,7 +10283,7 @@
     </row>
     <row r="59" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A59" s="2" t="s">
-        <v>231</v>
+        <v>177</v>
       </c>
       <c r="B59" s="2"/>
       <c r="C59" s="2" t="s">
@@ -10487,7 +10292,7 @@
       <c r="D59" t="s">
         <v>131</v>
       </c>
-      <c r="E59" s="41" t="s">
+      <c r="E59" s="2" t="s">
         <v>38</v>
       </c>
       <c r="F59" s="2">
@@ -10505,7 +10310,7 @@
     </row>
     <row r="60" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A60" s="2" t="s">
-        <v>232</v>
+        <v>177</v>
       </c>
       <c r="B60" s="2"/>
       <c r="C60" s="2" t="s">
@@ -10514,7 +10319,7 @@
       <c r="D60" t="s">
         <v>132</v>
       </c>
-      <c r="E60" s="41" t="s">
+      <c r="E60" s="2" t="s">
         <v>38</v>
       </c>
       <c r="F60" s="2">
@@ -10532,7 +10337,7 @@
     </row>
     <row r="61" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A61" s="2" t="s">
-        <v>233</v>
+        <v>177</v>
       </c>
       <c r="B61" s="2"/>
       <c r="C61" s="2" t="s">
@@ -10541,7 +10346,7 @@
       <c r="D61" t="s">
         <v>133</v>
       </c>
-      <c r="E61" s="41" t="s">
+      <c r="E61" s="2" t="s">
         <v>38</v>
       </c>
       <c r="F61" s="2">
@@ -10559,7 +10364,7 @@
     </row>
     <row r="62" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A62" s="2" t="s">
-        <v>234</v>
+        <v>177</v>
       </c>
       <c r="B62" s="2"/>
       <c r="C62" s="2" t="s">
@@ -10568,7 +10373,7 @@
       <c r="D62" t="s">
         <v>134</v>
       </c>
-      <c r="E62" s="41" t="s">
+      <c r="E62" s="2" t="s">
         <v>38</v>
       </c>
       <c r="F62" s="2">
@@ -10586,7 +10391,7 @@
     </row>
     <row r="63" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A63" s="2" t="s">
-        <v>235</v>
+        <v>177</v>
       </c>
       <c r="B63" s="2"/>
       <c r="C63" s="2" t="s">
@@ -10595,7 +10400,7 @@
       <c r="D63" t="s">
         <v>135</v>
       </c>
-      <c r="E63" s="41" t="s">
+      <c r="E63" s="2" t="s">
         <v>38</v>
       </c>
       <c r="F63" s="2">
@@ -10613,7 +10418,7 @@
     </row>
     <row r="64" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A64" s="2" t="s">
-        <v>236</v>
+        <v>177</v>
       </c>
       <c r="B64" s="2"/>
       <c r="C64" s="2" t="s">
@@ -10622,7 +10427,7 @@
       <c r="D64" t="s">
         <v>136</v>
       </c>
-      <c r="E64" s="41" t="s">
+      <c r="E64" s="2" t="s">
         <v>38</v>
       </c>
       <c r="F64" s="2">
@@ -10640,16 +10445,16 @@
     </row>
     <row r="65" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A65" s="2" t="s">
-        <v>237</v>
+        <v>177</v>
       </c>
       <c r="B65" s="2"/>
       <c r="C65" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="D65" s="43" t="s">
+      <c r="D65" s="12" t="s">
         <v>137</v>
       </c>
-      <c r="E65" s="41" t="s">
+      <c r="E65" s="2" t="s">
         <v>38</v>
       </c>
       <c r="F65" s="2">
@@ -10667,16 +10472,16 @@
     </row>
     <row r="66" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A66" s="2" t="s">
-        <v>238</v>
+        <v>177</v>
       </c>
       <c r="B66" s="2"/>
       <c r="C66" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="D66" s="43" t="s">
+      <c r="D66" s="12" t="s">
         <v>138</v>
       </c>
-      <c r="E66" s="41" t="s">
+      <c r="E66" s="2" t="s">
         <v>38</v>
       </c>
       <c r="F66" s="2">
@@ -10694,16 +10499,16 @@
     </row>
     <row r="67" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A67" s="2" t="s">
-        <v>239</v>
+        <v>177</v>
       </c>
       <c r="B67" s="2"/>
       <c r="C67" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="D67" s="43" t="s">
+      <c r="D67" s="12" t="s">
         <v>139</v>
       </c>
-      <c r="E67" s="41" t="s">
+      <c r="E67" s="2" t="s">
         <v>38</v>
       </c>
       <c r="F67" s="2">
@@ -10721,16 +10526,16 @@
     </row>
     <row r="68" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A68" s="2" t="s">
-        <v>240</v>
+        <v>177</v>
       </c>
       <c r="B68" s="2"/>
       <c r="C68" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="D68" s="43" t="s">
+      <c r="D68" s="12" t="s">
         <v>140</v>
       </c>
-      <c r="E68" s="41" t="s">
+      <c r="E68" s="2" t="s">
         <v>38</v>
       </c>
       <c r="F68" s="2">
@@ -10748,13 +10553,13 @@
     </row>
     <row r="69" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A69" s="2" t="s">
-        <v>241</v>
+        <v>177</v>
       </c>
       <c r="B69" s="2"/>
       <c r="C69" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="D69" s="43" t="s">
+      <c r="D69" s="12" t="s">
         <v>149</v>
       </c>
       <c r="E69" s="2" t="s">
@@ -10775,7 +10580,7 @@
     </row>
     <row r="70" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A70" s="2" t="s">
-        <v>242</v>
+        <v>177</v>
       </c>
       <c r="B70" s="2"/>
       <c r="C70" s="2" t="s">
@@ -10802,7 +10607,7 @@
     </row>
     <row r="71" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A71" s="2" t="s">
-        <v>243</v>
+        <v>177</v>
       </c>
       <c r="B71" s="2"/>
       <c r="C71" s="2" t="s">
@@ -10829,7 +10634,7 @@
     </row>
     <row r="72" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A72" s="2" t="s">
-        <v>244</v>
+        <v>177</v>
       </c>
       <c r="B72" s="2"/>
       <c r="C72" s="2" t="s">
@@ -10856,7 +10661,7 @@
     </row>
     <row r="73" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A73" s="2" t="s">
-        <v>245</v>
+        <v>177</v>
       </c>
       <c r="B73" s="2"/>
       <c r="C73" s="2" t="s">
@@ -10882,55 +10687,55 @@
       </c>
     </row>
     <row r="74" spans="1:9" ht="29" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A74" s="45" t="s">
+      <c r="A74" s="47" t="s">
         <v>176</v>
       </c>
-      <c r="B74" s="46"/>
-      <c r="C74" s="46"/>
-      <c r="D74" s="46"/>
-      <c r="E74" s="46"/>
-      <c r="F74" s="46"/>
-      <c r="G74" s="46"/>
-      <c r="H74" s="46"/>
-      <c r="I74" s="46"/>
-    </row>
-    <row r="75" spans="1:9" ht="46" x14ac:dyDescent="0.2">
-      <c r="A75" s="47" t="s">
+      <c r="B74" s="48"/>
+      <c r="C74" s="48"/>
+      <c r="D74" s="48"/>
+      <c r="E74" s="48"/>
+      <c r="F74" s="48"/>
+      <c r="G74" s="48"/>
+      <c r="H74" s="48"/>
+      <c r="I74" s="48"/>
+    </row>
+    <row r="75" spans="1:9" ht="49" x14ac:dyDescent="0.2">
+      <c r="A75" s="13" t="s">
         <v>24</v>
       </c>
-      <c r="B75" s="47" t="s">
+      <c r="B75" s="13" t="s">
         <v>41</v>
       </c>
-      <c r="C75" s="47" t="s">
+      <c r="C75" s="13" t="s">
         <v>26</v>
       </c>
-      <c r="D75" s="47" t="s">
+      <c r="D75" s="13" t="s">
         <v>15</v>
       </c>
-      <c r="E75" s="47" t="s">
+      <c r="E75" s="13" t="s">
         <v>31</v>
       </c>
-      <c r="F75" s="47" t="s">
+      <c r="F75" s="13" t="s">
         <v>21</v>
       </c>
-      <c r="G75" s="47" t="s">
+      <c r="G75" s="13" t="s">
         <v>27</v>
       </c>
-      <c r="H75" s="47" t="s">
+      <c r="H75" s="13" t="s">
         <v>22</v>
       </c>
-      <c r="I75" s="47" t="s">
+      <c r="I75" s="13" t="s">
         <v>23</v>
       </c>
     </row>
     <row r="76" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A76" s="48"/>
-      <c r="B76" s="49"/>
+      <c r="A76" s="14"/>
+      <c r="B76" s="15"/>
       <c r="C76" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="D76" s="42" t="s">
-        <v>141</v>
+      <c r="D76" s="52" t="s">
+        <v>178</v>
       </c>
       <c r="E76" s="2" t="s">
         <v>16</v>
@@ -10949,13 +10754,13 @@
       </c>
     </row>
     <row r="77" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A77" s="50"/>
-      <c r="B77" s="51"/>
+      <c r="A77" s="16"/>
+      <c r="B77" s="17"/>
       <c r="C77" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="D77" s="42" t="s">
-        <v>142</v>
+      <c r="D77" s="11" t="s">
+        <v>141</v>
       </c>
       <c r="E77" s="2" t="s">
         <v>16</v>
@@ -10970,17 +10775,17 @@
         <v>4</v>
       </c>
       <c r="I77" s="2" t="s">
-        <v>36</v>
+        <v>19</v>
       </c>
     </row>
     <row r="78" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A78" s="52"/>
-      <c r="B78" s="53"/>
+      <c r="A78" s="18"/>
+      <c r="B78" s="19"/>
       <c r="C78" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="D78" s="42" t="s">
-        <v>143</v>
+      <c r="D78" s="11" t="s">
+        <v>142</v>
       </c>
       <c r="E78" s="2" t="s">
         <v>16</v>
@@ -11004,8 +10809,8 @@
       <c r="C79" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="D79" s="42" t="s">
-        <v>144</v>
+      <c r="D79" s="11" t="s">
+        <v>143</v>
       </c>
       <c r="E79" s="2" t="s">
         <v>16</v>
@@ -11029,8 +10834,8 @@
       <c r="C80" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="D80" s="42" t="s">
-        <v>145</v>
+      <c r="D80" s="11" t="s">
+        <v>144</v>
       </c>
       <c r="E80" s="2" t="s">
         <v>16</v>
@@ -11054,8 +10859,8 @@
       <c r="C81" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="D81" s="42" t="s">
-        <v>146</v>
+      <c r="D81" s="11" t="s">
+        <v>145</v>
       </c>
       <c r="E81" s="2" t="s">
         <v>16</v>
@@ -11079,8 +10884,8 @@
       <c r="C82" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="D82" s="2" t="s">
-        <v>16</v>
+      <c r="D82" s="11" t="s">
+        <v>146</v>
       </c>
       <c r="E82" s="2" t="s">
         <v>16</v>
@@ -11095,7 +10900,7 @@
         <v>4</v>
       </c>
       <c r="I82" s="2" t="s">
-        <v>16</v>
+        <v>36</v>
       </c>
     </row>
     <row r="83" spans="1:9" x14ac:dyDescent="0.2">
@@ -11329,7 +11134,7 @@
       <c r="C92" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="D92" s="42" t="s">
+      <c r="D92" s="11" t="s">
         <v>147</v>
       </c>
       <c r="E92" s="2" t="s">
@@ -11354,7 +11159,7 @@
       <c r="C93" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="D93" s="42" t="s">
+      <c r="D93" s="11" t="s">
         <v>148</v>
       </c>
       <c r="E93" s="2" t="s">
@@ -12143,7 +11948,7 @@
       <c r="A150" s="2"/>
       <c r="B150" s="2"/>
       <c r="C150" s="2"/>
-      <c r="E150" s="41"/>
+      <c r="E150" s="2"/>
       <c r="F150" s="2"/>
       <c r="G150" s="2"/>
       <c r="H150" s="2"/>
@@ -12153,7 +11958,7 @@
       <c r="A151" s="2"/>
       <c r="B151" s="2"/>
       <c r="C151" s="2"/>
-      <c r="E151" s="41"/>
+      <c r="E151" s="2"/>
       <c r="F151" s="2"/>
       <c r="G151" s="2"/>
       <c r="H151" s="2"/>
@@ -12163,7 +11968,7 @@
       <c r="A152" s="2"/>
       <c r="B152" s="2"/>
       <c r="C152" s="2"/>
-      <c r="E152" s="41"/>
+      <c r="E152" s="2"/>
       <c r="F152" s="2"/>
       <c r="G152" s="2"/>
       <c r="H152" s="2"/>
@@ -12173,7 +11978,7 @@
       <c r="A153" s="2"/>
       <c r="B153" s="2"/>
       <c r="C153" s="2"/>
-      <c r="E153" s="41"/>
+      <c r="E153" s="2"/>
       <c r="F153" s="2"/>
       <c r="G153" s="2"/>
       <c r="H153" s="2"/>
@@ -12183,7 +11988,7 @@
       <c r="A154" s="2"/>
       <c r="B154" s="2"/>
       <c r="C154" s="2"/>
-      <c r="E154" s="41"/>
+      <c r="E154" s="2"/>
       <c r="F154" s="2"/>
       <c r="G154" s="2"/>
       <c r="H154" s="2"/>
@@ -12193,7 +11998,7 @@
       <c r="A155" s="2"/>
       <c r="B155" s="2"/>
       <c r="C155" s="2"/>
-      <c r="E155" s="41"/>
+      <c r="E155" s="2"/>
       <c r="F155" s="2"/>
       <c r="G155" s="2"/>
       <c r="H155" s="2"/>
@@ -12203,7 +12008,7 @@
       <c r="A156" s="2"/>
       <c r="B156" s="2"/>
       <c r="C156" s="2"/>
-      <c r="E156" s="41"/>
+      <c r="E156" s="2"/>
       <c r="F156" s="2"/>
       <c r="G156" s="2"/>
       <c r="H156" s="2"/>
@@ -12213,7 +12018,7 @@
       <c r="A157" s="2"/>
       <c r="B157" s="2"/>
       <c r="C157" s="2"/>
-      <c r="E157" s="41"/>
+      <c r="E157" s="2"/>
       <c r="F157" s="2"/>
       <c r="G157" s="2"/>
       <c r="H157" s="2"/>
@@ -12223,7 +12028,7 @@
       <c r="A158" s="2"/>
       <c r="B158" s="2"/>
       <c r="C158" s="2"/>
-      <c r="E158" s="41"/>
+      <c r="E158" s="2"/>
       <c r="F158" s="2"/>
       <c r="G158" s="2"/>
       <c r="H158" s="2"/>
@@ -12233,7 +12038,7 @@
       <c r="A159" s="2"/>
       <c r="B159" s="2"/>
       <c r="C159" s="2"/>
-      <c r="E159" s="41"/>
+      <c r="E159" s="2"/>
       <c r="F159" s="2"/>
       <c r="G159" s="2"/>
       <c r="H159" s="2"/>
@@ -12243,7 +12048,7 @@
       <c r="A160" s="2"/>
       <c r="B160" s="2"/>
       <c r="C160" s="2"/>
-      <c r="E160" s="41"/>
+      <c r="E160" s="2"/>
       <c r="F160" s="2"/>
       <c r="G160" s="2"/>
       <c r="H160" s="2"/>
@@ -12253,7 +12058,7 @@
       <c r="A161" s="2"/>
       <c r="B161" s="2"/>
       <c r="C161" s="2"/>
-      <c r="E161" s="41"/>
+      <c r="E161" s="2"/>
       <c r="F161" s="2"/>
       <c r="G161" s="2"/>
       <c r="H161" s="2"/>
@@ -12263,7 +12068,7 @@
       <c r="A162" s="2"/>
       <c r="B162" s="2"/>
       <c r="C162" s="2"/>
-      <c r="E162" s="41"/>
+      <c r="E162" s="2"/>
       <c r="F162" s="2"/>
       <c r="G162" s="2"/>
       <c r="H162" s="2"/>
@@ -12273,7 +12078,7 @@
       <c r="A163" s="2"/>
       <c r="B163" s="2"/>
       <c r="C163" s="2"/>
-      <c r="E163" s="41"/>
+      <c r="E163" s="2"/>
       <c r="F163" s="2"/>
       <c r="G163" s="2"/>
       <c r="H163" s="2"/>
@@ -12283,7 +12088,7 @@
       <c r="A164" s="2"/>
       <c r="B164" s="2"/>
       <c r="C164" s="2"/>
-      <c r="E164" s="41"/>
+      <c r="E164" s="2"/>
       <c r="F164" s="2"/>
       <c r="G164" s="2"/>
       <c r="H164" s="2"/>
@@ -12293,7 +12098,7 @@
       <c r="A165" s="2"/>
       <c r="B165" s="2"/>
       <c r="C165" s="2"/>
-      <c r="E165" s="41"/>
+      <c r="E165" s="2"/>
       <c r="F165" s="2"/>
       <c r="G165" s="2"/>
       <c r="H165" s="2"/>
@@ -12303,7 +12108,7 @@
       <c r="A166" s="2"/>
       <c r="B166" s="2"/>
       <c r="C166" s="2"/>
-      <c r="D166" s="43"/>
+      <c r="D166" s="12"/>
       <c r="E166" s="2"/>
       <c r="F166" s="2"/>
       <c r="G166" s="2"/>

</xml_diff>